<commit_message>
PRODESP-DER: aba de discovery Service Cloud/CTI (atendimento geral + gestao de chamados)
Fato novo: DER quer tambem atendimento geral com CTI/URA (fornecedor
desconhecido), agentes humanos, agente de IA coworker, canais Omni-Channel,
niveis de atendimento, turnos, roteamento, volumetria e SLA. Perguntas
grounded em 10 atomos da KB central, incluindo alerta sobre a descontinuacao
da Open CTI (retirada fev/2028) em favor do Salesforce Voice.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Scopezilla/PRODESP-DER/outputs/scoping-deliverables.xlsx
+++ b/Scopezilla/PRODESP-DER/outputs/scoping-deliverables.xlsx
@@ -11,17 +11,19 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery - MVP Emergencial" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery - Field Service Ind." sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery - Agentforce WhatsApp" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery - Setor Público" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscos" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap - Catalogo DER" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery - Service Cloud CTI" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discovery - Setor Público" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap - Catalogo DER" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Discovery - MVP Emergencial'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Discovery - Field Service Ind.'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Discovery - Agentforce WhatsApp'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Discovery - Setor Público'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Riscos'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Roadmap - Catalogo DER'!$A$4:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Discovery - Service Cloud CTI'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Discovery - Setor Público'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Riscos'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Roadmap - Catalogo DER'!$A$4:$F$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -522,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -545,7 +547,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Gerado em 09/09/2026 16:01 — Scopezilla / PRODESP-DER</t>
+          <t>Gerado em 09/09/2026 16:33 — Scopezilla / PRODESP-DER</t>
         </is>
       </c>
     </row>
@@ -600,36 +602,43 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>4. Discovery — Setor Público (padrão): bloco de perguntas que aplicamos em todo projeto de setor público (governança, LGPD, licitação, acessibilidade, integração com outros órgãos, continuidade de serviço essencial).</t>
+          <t>4. Discovery — Service Cloud / CTI: fato novo — o DER também quer um atendimento geral com gestão de chamados (Service Cloud), incluindo agentes humanos, agente de IA coworker, canais no Omni-Channel, níveis de atendimento, turnos, regras de roteamento, volumetria, SLA e a integração de CTI com a URA do DER (URA ainda não identificada — a aba já traz o alinhamento necessário sobre a descontinuação da Open CTI pela Salesforce).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>5. Riscos: matriz de risco potencial com pergunta de validação para cada risco — cobre os riscos já citados na POC (matriz de risco por cenário, alarme de 5 min) e riscos adicionais de escala, dados e governança.</t>
+          <t>5. Discovery — Setor Público (padrão): bloco de perguntas que aplicamos em todo projeto de setor público (governança, LGPD, licitação, acessibilidade, integração com outros órgãos, continuidade de serviço essencial).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>6. Roadmap — Catálogo DER: mapeamento indicativo de TODOS os serviços listados na Carta de Serviços do DER-SP, agrupados em ondas de discussão a partir do MVP (atendimento emergencial). É um mapa de discussão para orientar o roadmap, não um cronograma comprometido — sequenciamento, prazos e equipe são definidos depois, com as skills de roadmap/estimate.</t>
+          <t>6. Riscos: matriz de risco potencial com pergunta de validação para cada risco — cobre os riscos já citados na POC (matriz de risco por cenário, alarme de 5 min) e riscos adicionais de escala, dados e governança.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>7. Roadmap — Catálogo DER: mapeamento indicativo de TODOS os serviços listados na Carta de Serviços do DER-SP, agrupados em ondas de discussão a partir do MVP (atendimento emergencial). É um mapa de discussão para orientar o roadmap, não um cronograma comprometido — sequenciamento, prazos e equipe são definidos depois, com as skills de roadmap/estimate.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>LEGENDA</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>'Confirmado na POC' = a POC já responde isso explicitamente. 'A validar' = a POC assume ou não define; precisa confirmação do DER na sessão. 'Gap' = não aparece na POC e é um ponto novo a explorar.</t>
         </is>
@@ -2241,6 +2250,859 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Bloco</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Pergunta de Discovery</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Por que perguntamos</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Referência / Caso de uso padrão</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Resposta do DER (sessão)</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>A. Escopo do Atendimento Geral e Gestão de Chamados</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Esse novo atendimento (fato novo, distinto do atendimento emergencial em rodovia) é para o público externo (cidadão), interno (servidores do DER), ou ambos?</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Define se é Service Cloud voltado a Customer Service, Employee Service, ou os dois — com filas, canais e SLA potencialmente distintos para cada público.</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr"/>
+      <c r="E3" s="9" t="inlineStr"/>
+      <c r="F3" s="9" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Quais tipos de solicitação esse atendimento deve cobrir — dúvidas sobre os serviços do catálogo do DER (multas, autorizações), reclamações de infraestrutura viária, pedidos de informação (LAI/SIC), ou é um canal único que hoje está fragmentado entre Ouvidoria, SIC e atendimento telefônico?</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>A Carta de Serviços do DER já lista Ouvidoria e SIC como canais formais existentes — se este projeto cobre o mesmo escopo, é preciso decidir se substitui, integra ou complementa esses canais institucionais, para não criar canal duplicado.</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr"/>
+      <c r="E4" s="9" t="inlineStr"/>
+      <c r="F4" s="9" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Existe hoje algum sistema de gestão de chamados (ticket, planilha, e-mail, ou mesmo processo manual) que será substituído, e há necessidade de migrar histórico de chamados abertos?</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>Determina o escopo de migração de dados e o período de transição/paralelo entre o sistema atual e o novo atendimento.</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr"/>
+      <c r="E5" s="9" t="inlineStr"/>
+      <c r="F5" s="9" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Um chamado deste atendimento geral pode se relacionar com uma ocorrência do atendimento emergencial de rodovia (ex: um sinistro que gera depois uma reclamação formal)? Se sim, precisa haver vínculo/rastreabilidade entre os dois?</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Afeta o modelo de dados — se o Case deste atendimento e a Ocorrência do Field Service (POC emergencial) compartilham o mesmo Contato/Conta e precisam de link cruzado para visão única do cidadão.</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr"/>
+      <c r="F6" s="9" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>B. Agentes Humanos de Atendimento</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Quantos agentes humanos estão previstos para esse atendimento, e eles são servidores do próprio DER, terceirizados, ou a mesma central que hoje atende o C2C do atendimento emergencial?</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Determina licenciamento de usuários e se a força de trabalho é compartilhada com o C2C (visto na POC) ou é equipe nova e separada — mudam o desenho de filas e de capacidade.</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr"/>
+      <c r="F8" s="9" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Os agentes atuam de forma generalista (qualquer chamado) ou especializados por assunto (ex: multas, autorizações, infraestrutura)? Essa estrutura de equipe já existe hoje, mesmo informalmente?</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>A estrutura de equipe real de hoje é o insumo para decidir entre roteamento por fila única ou por habilidades (skills-based) — não é uma escolha a ser feita no vácuo.</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>[KA-4393] Omni-Channel: Skills-Based vs Queue-Based Routing</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr"/>
+      <c r="F9" s="9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Qual o nível de familiaridade da equipe com ferramentas de atendimento digital (console de CRM, sistemas de chamado)? É a primeira vez usando uma ferramenta desse tipo?</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Afeta diretamente o esforço de capacitação/change management e o quão guiada a interface do console precisa ser desenhada.</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr"/>
+      <c r="F10" s="9" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Existe hoje alguma meta de produtividade por agente (chamados/dia, tempo médio de atendimento) usada para dimensionar a equipe atual?</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>Insumo real de capacidade operacional para o desenho de Presence Configuration do Omni-Channel — não serve para estimar headcount aqui (isso é do skill `estimate`), serve para entender a realidade da operação.</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr"/>
+      <c r="E11" s="9" t="inlineStr"/>
+      <c r="F11" s="9" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>C. Agente de IA Coworker (Agentforce)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>O 'agente de IA coworker' deve assistir o agente humano (sugerir resposta, resumir o caso, buscar na base de conhecimento) ou atuar de forma autônoma atendendo diretamente o cidadão/servidor antes de escalar para humano?</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>São dois produtos/casos de uso distintos dentro da marca Agentforce: o Coworker é posicionado como ponto de entrada em linguagem natural dentro do CRM (busca e síntese); um agente autônomo de atendimento direto ao usuário externo é outro desenho (Agentforce Service Agent). A resposta muda a arquitetura inteira.</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>[KA-18840] Agentforce Coworker — Benefits and Core Use Cases</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Se for um agente autônomo atendendo diretamente o cidadão: em quais canais ele atua primeiro (o mesmo WhatsApp do atendimento emergencial, um chat no site, outro), e qual o critério de handoff para um agente humano?</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Reaproveita o mesmo desenho de guardrails de escopo já necessário no Agentforce do MVP emergencial, mas aqui o domínio é diferente (chamados administrativos, não emergência viária) — o agente precisa de outro conjunto de tópicos/ações.</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr"/>
+      <c r="E14" s="9" t="inlineStr"/>
+      <c r="F14" s="9" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Se for um 'coworker' assistindo o agente humano: quais fontes de conhecimento ele deve consultar — Knowledge do Salesforce, base de conhecimento do DER hoje em outro sistema, dados de CRM/Data Cloud?</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Sem fonte de conhecimento indexada, o coworker não tem o que sintetizar — a Busca Empresarial Agêntica exige Knowledge configurado e Search Manager antes de funcionar.</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>[KA-12172] Agentic Enterprise Search for Agentforce Service Agent</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr"/>
+      <c r="F15" s="9" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Existe hoje uma base de conhecimento/FAQ estruturada (mesmo informal) sobre os serviços do DER que possa alimentar esse agente, ou isso também precisa ser construído do zero?</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Base de conhecimento é pré-requisito técnico da Busca Empresarial Agêntica, não só uma questão de UX — sem isso não há o que o coworker buscar e sintetizar.</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>[KA-12172]</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr"/>
+      <c r="F16" s="9" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>D. Canais Habilitados no Omni-Channel</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Quais canais o DER quer habilitar no Omni-Channel para este atendimento geral — voz/telefone, WhatsApp, chat no site, e-mail, redes sociais? É a mesma lista de canais do atendimento emergencial ou um conjunto diferente?</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Cada canal tem pré-requisito de licenciamento e configuração próprio (voz depende diretamente da decisão de CTI no bloco J) — sem essa lista fechada não se desenha o roteamento nem a capacidade dos agentes.</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr"/>
+      <c r="E18" s="9" t="inlineStr"/>
+      <c r="F18" s="9" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Cada canal terá o mesmo grupo de agentes atendendo em fila compartilhada, ou equipes dedicadas por canal (ex: equipe de voz separada da equipe de chat/WhatsApp)?</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Define se a capacidade (Presence Configuration) é única e compartilhada entre canais ou segmentada — impacta diretamente a regra de roteamento do bloco G.</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr"/>
+      <c r="E19" s="9" t="inlineStr"/>
+      <c r="F19" s="9" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Há alguma restrição de licenciamento ou integração legada que force o uso do Omni-Channel Standard, ou o DER está aberto à recomendação padrão da Salesforce de usar o Enhanced Omni-Channel?</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>O Enhanced Omni-Channel é a recomendação padrão da Salesforce e suporta capacidades (como reatribuição de trabalho) que o Standard não tem — vale confirmar cedo, pois muda a experiência do agente.</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>[KA-4401] Choose Enhanced Omni-Channel over Standard</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr"/>
+      <c r="F20" s="9" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>E. Níveis de Atendimento (Tiers) e Escalonamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Quantos níveis de atendimento o DER quer operar (ex: 1ª linha / especialista / backoffice, ou N1/N2/N3), e o que caracteriza a passagem de um chamado de um nível para o outro?</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Estrutura de tiers direciona diretamente o desenho de filas/habilidades e das regras de escalonamento — é o núcleo do que foi pedido explicitamente para este discovery.</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr"/>
+      <c r="E22" s="9" t="inlineStr"/>
+      <c r="F22" s="9" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Hoje, mesmo fora de sistema, existe alguma prática de escalonamento por tipo de assunto ou por tempo sem resposta?</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>As Regras de Escalonamento do Service Cloud automatizam esse comportamento (idade do caso, reatribuição automática, notificação) — mas a regra de negócio real precisa vir do processo já praticado pelo DER, nunca ser inventada.</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>[KA-4453] Configure Case Escalation Actions · [KA-4455] Configure Case Escalation Rules</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr"/>
+      <c r="F23" s="9" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Para assuntos que exigem múltiplos especialistas simultâneos (ex: um chamado que envolve jurídico e engenharia ao mesmo tempo), o modelo esperado é hierárquico (sobe de nível) ou colaborativo (várias áreas trabalham juntas no mesmo caso)?</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Se colaborativo, um modelo de colaboração sem tiers rígidos, orientado a especialistas, pode ser mais aderente do que uma escada tradicional de níveis — vale perguntar antes de assumir hierarquia como padrão.</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>[KA-4549] Service Swarming Overview and Collaboration Modes</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr"/>
+      <c r="F24" s="9" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>F. Turnos e Horário de Atendimento</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Qual o horário de atendimento previsto (comercial, estendido, 24x7), e ele é igual para todos os canais e tipos de chamado, ou varia (ex: voz só em horário comercial, WhatsApp mais estendido)?</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>O horário de atendimento configurado no Service Cloud alimenta diretamente o cálculo de SLA/Marcos e as regras de escalonamento — precisa ser definido por canal/fila, não assumido como valor único.</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>[KA-3976] Configure and Apply Business Hours for Cases, Escalations, Entitlements, and Milestones</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr"/>
+      <c r="F26" s="9" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Existem turnos de trabalho definidos hoje para a equipe (ex: manhã/tarde, plantão), e como a troca de turno afeta um chamado em andamento (transferência de responsabilidade)?</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Turno não é um conceito único nativo do Service Cloud — normalmente é refletido combinando Presence Configuration e Horário de Atendimento; a regra de handoff entre turnos é do negócio do DER e precisa ser levantada, não assumida.</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr"/>
+      <c r="E27" s="9" t="inlineStr"/>
+      <c r="F27" s="9" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n">
+        <v>21</v>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Feriados e pontos facultativos do calendário público estadual afetam o horário de atendimento (ex: SLA pausa nesses dias)?</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>O recurso de Horário de Atendimento do Salesforce suporta calendário de feriados vinculado — pergunta prática para não gerar cálculo de SLA incorreto em dia sem expediente.</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>[KA-3976]</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr"/>
+      <c r="F28" s="9" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>G. Regras de Roteamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>O roteamento de um chamado para o agente certo deve ser por fila simples (qualquer agente da fila atende) ou por habilidades específicas (ex: só quem sabe de 'autorização especial de transporte' recebe esse chamado)?</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>É a decisão central de arquitetura de roteamento do Omni-Channel: fila é mais simples de manter; habilidades é mais preciso, mas exige mapear e manter o cadastro de skills por agente.</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>[KA-4393] Omni-Channel: Skills-Based vs Queue-Based Routing</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr"/>
+      <c r="F30" s="9" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Dentro de uma mesma fila/habilidade, quando dois chamados chegam ao mesmo tempo e há um agente livre, o critério de prioridade deve ser 'quem está livre há mais tempo' ou 'quem está menos ocupado no momento'?</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>O Omni-Channel oferece os modelos 'Least Active' e 'Most Available' — decisão de negócio que muda a distribuição de carga entre agentes; não tem resposta única certa, precisa ser escolhida pelo DER.</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>[KA-4539] Omni-Channel routing model selection: Least Active vs Most Available</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr"/>
+      <c r="F31" s="9" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Há previsão de usar classificação automática por IA para direcionar o chamado à fila certa, ou a classificação inicial será sempre manual/definida pelo próprio canal de abertura?</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>O Einstein Case Routing conecta a classificação automática de caso à lógica de roteamento já configurada — só é viável se já existir roteamento por fila/habilidade configurado por trás; não substitui essa decisão, depende dela.</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>[KA-4339] Einstein Case Routing: Built-in vs. Custom/External Routing</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr"/>
+      <c r="F32" s="9" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>H. Volumetria</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Qual o volume estimado de chamados/contatos por mês (ou por dia) para esse atendimento geral — mesmo que seja uma estimativa aproximada baseada no volume atual de Ouvidoria, SIC ou telefone?</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Volumetria real é o insumo que dimensiona capacidade de fila, número de agentes e viabilidade de metas de SLA — sem isso, todo o resto do desenho de atendimento fica no vácuo.</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr"/>
+      <c r="E34" s="9" t="inlineStr"/>
+      <c r="F34" s="9" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Esse volume tem sazonalidade ou pico conhecido (ex: período de vencimento de multas, época de chuva, campanha de comunicação do DER)?</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Pico sazonal pressiona diretamente a capacidade do Omni-Channel e o cumprimento de SLA — mesmo racional já levantado para o Field Service, aqui aplicado ao atendimento geral.</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr"/>
+      <c r="E35" s="9" t="inlineStr"/>
+      <c r="F35" s="9" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n">
+        <v>27</v>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Qual a proporção esperada entre canais (ex: hoje X% por telefone, Y% por e-mail)? Isso já é medido em algum relatório de Ouvidoria/SIC hoje?</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Sem essa distribuição por canal, a capacidade de cada canal (voz exige presença dedicada; chat permite atendimento simultâneo) fica sem base real para dimensionamento.</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr"/>
+      <c r="E36" s="9" t="inlineStr"/>
+      <c r="F36" s="9" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>I. SLA / Entitlements / Milestones</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Existe hoje algum SLA formal (mesmo que apenas normativo, fora de sistema) de prazo de resposta e de resolução por tipo de chamado ou por nível de atendimento?</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>As políticas de SLA do Service Cloud são estruturadas como marcos dentro de um prazo — sem meta real definida pelo DER, a configuração fica arbitrária e sem valor de negócio.</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>[KA-4033] SLA Policies for Entitlements · [KA-4590] SLA Policies (Entitlement Process) Overview</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr"/>
+      <c r="F38" s="9" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>O SLA de resposta/resolução precisa ser diferenciado por tipo de solicitante (cidadão comum vs. outro órgão público vs. imprensa) ou é uniforme para todos?</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="inlineStr">
+        <is>
+          <t>A Gestão de Direitos (Entitlement Management) do Service Cloud foi desenhada justamente para dar 'o nível de suporte prometido' por perfil — pergunta chave para saber se um único SLA Policy basta ou se são necessários vários.</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr"/>
+      <c r="E39" s="9" t="inlineStr"/>
+      <c r="F39" s="9" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Quem será o responsável por tratar os marcos de SLA que não se fecham automaticamente quando a condição de negócio é cumprida?</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Marcos (Milestones) não se completam automaticamente sem automação (Flow/Apex) — é um gap frequente em desenhos de entitlement; vale sinalizar desde já que alguém vai precisar ser o dono desse processo.</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>[KA-0463] Do not expect entitlement Milestones to auto-complete without automation</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr"/>
+      <c r="F40" s="9" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="B41" s="9" t="inlineStr">
+        <is>
+          <t>Há diferenciação de SLA por gravidade/prioridade do assunto (semelhante à matriz de risco usada no atendimento emergencial), ou o SLA aqui é só por prazo corrido/tipo de assunto?</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="inlineStr">
+        <is>
+          <t>Conecta com o racional já usado na POC de emergência — mas aqui é atendimento administrativo, então a variável de 'gravidade' muda de sentido (ex: reclamação grave de segurança viária x dúvida simples de documentação).</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr"/>
+      <c r="E41" s="9" t="inlineStr"/>
+      <c r="F41" s="9" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>J. CTI / Telefonia / URA</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n">
+        <v>32</v>
+      </c>
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>Qual é hoje o sistema de URA/telefonia do DER (fornecedor, se é PABX próprio, solução em nuvem, ou terceirizado)? Mesmo sem saber o nome exato agora, quem no DER saberia informar (TI, fornecedor de telefonia, área de atendimento)?</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="inlineStr">
+        <is>
+          <t>É a pergunta mais crítica deste bloco — sem saber qual sistema é, não é possível avaliar se a integração é tecnicamente viável nem por qual caminho.</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr"/>
+      <c r="E43" s="9" t="inlineStr"/>
+      <c r="F43" s="9" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Alinhamento importante antes de prosseguir: a Salesforce está descontinuando a Open CTI (a API clássica de integração com URA/PABX de terceiros) — retirada prevista para fevereiro de 2028 e já indisponível para novos orgs Agentforce Service; o caminho recomendado pela própria Salesforce é migrar para o Salesforce Voice (voz nativa da plataforma). Dado isso, o DER prefere manter a URA/PABX atual integrada via CTI de terceiro (se ainda viável), ou está aberto a avaliar o Salesforce Voice como solução de voz nativa?</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>Essa é uma decisão arquitetural que muda o projeto inteiro de voz — precisa ser surfaceada agora, antes que 'vamos integrar com a URA deles' seja tratado como premissa fechada de escopo.</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>[KA-5474] Open CTI vs Salesforce Voice vs Sales Dialer · [KA-5475]/[KA-5427] Avoid new implementations on Open CTI (retiring Feb 2028)</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr"/>
+      <c r="F44" s="9" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n">
+        <v>34</v>
+      </c>
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>Se a URA atual precisar ser mantida (ex: contrato vigente com fornecedor de telefonia, integração com outros sistemas do DER), já existe confirmação de que o fornecedor da URA oferece uma API de CTI compatível?</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="inlineStr">
+        <is>
+          <t>Mesmo dentro da Open CTI existem APIs diferentes e não intercambiáveis entre Salesforce Classic e Lightning — a viabilidade técnica depende de o fornecedor de telefonia suportar a API certa; isso não é dado adquirido, precisa ser confirmado com o fornecedor.</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>[KA-5435] Select the correct Open CTI API (Classic vs Lightning) · [KA-5429]</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr"/>
+      <c r="F45" s="9" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>Existe contrato vigente com o fornecedor de telefonia/URA com prazo de vigência relevante para a decisão entre manter a integração via CTI de terceiro ou migrar para o Salesforce Voice?</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>A decisão de arquitetura de voz tem também uma dimensão contratual/comercial que pode pesar mais que a técnica — vale levantar já no discovery para não travar o projeto depois.</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr"/>
+      <c r="E46" s="9" t="inlineStr"/>
+      <c r="F46" s="9" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="n">
+        <v>36</v>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
+        <is>
+          <t>O atendimento por voz (seja qual for a solução escolhida) precisa gravar chamadas, transcrever automaticamente, ou gerar algum registro/auditoria específica por exigência de órgão público?</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="inlineStr">
+        <is>
+          <t>Gravação/transcrição pode ser requisito de compliance de setor público — mas aqui especificamente também muda a escolha entre Open CTI (tipicamente sem gravação nativa, depende do fornecedor terceiro) e Salesforce Voice (com transcrição/gravação nativas).</t>
+        </is>
+      </c>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>[KA-9528] Public Sector — Security Setup Overview</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr"/>
+      <c r="F47" s="9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <mergeCells count="10">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A21:F21"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A25:F25"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2568,7 +3430,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2943,7 +3805,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>